<commit_message>
Confirm 54 repository PDFs in worker briefs
</commit_message>
<xml_diff>
--- a/project-admin/PDF_Inventory_and_Worker_Assignments.xlsx
+++ b/project-admin/PDF_Inventory_and_Worker_Assignments.xlsx
@@ -488,12 +488,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Expected-count discrepancy</t>
+          <t>Confirmed scope</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>User reports 55 additional repo PDFs; current main branch clone contains 54. One file not yet located.</t>
+          <t>54 repo PDFs / 2,128 pages confirmed; plus 12 attached Sequence &amp; Series PDFs / 496 pages = 66 PDFs / 2,624 pages. No additional repo PDF is expected at this time.</t>
         </is>
       </c>
     </row>

</xml_diff>